<commit_message>
chore: add tools, update tracker/progress, expand gitignore
- Add tools/analyze_line_stop.py and tools/validate_build.py
- Update PX4_DXP_Tracker.xlsx and docs/Progress/PROGRESS.md
- Gitignore local-only dirs: Encoder_Fix/, PX4_params/, Simple Demo/,
  docs/Architecture/, docs/TODO/, image_ref/, tools/rosbag.txt

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PX4_DXP_Tracker.xlsx
+++ b/PX4_DXP_Tracker.xlsx
@@ -5084,7 +5084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="44.6640625" customWidth="1" min="1" max="1"/>
@@ -6617,44 +6617,38 @@
           <t>RPP Controller</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>Latency (P2.4)</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
-        <is>
-          <t>use_imu_extrapolation</t>
-        </is>
-      </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="E35" s="15" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="F35" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I35" s="7" t="inlineStr">
-        <is>
-          <t>Enable velocity-based pose extrapolation</t>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Tracking Profile</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>segment_stop_yaw_rate_threshold</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>rad/s</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>CORNER_STOP yaw-rate floor — rover must rotate &lt;this (with speed floor) for dwell before pivot (BUG-T1 036f116)</t>
         </is>
       </c>
     </row>
@@ -6666,12 +6660,12 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Latency (P2.4)</t>
+          <t>Tracking Profile</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>imu_max_extrap_age_s</t>
+          <t>segment_align_settle_s</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
@@ -6679,20 +6673,14 @@
           <t>float</t>
         </is>
       </c>
-      <c r="E36" s="16" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="F36" s="16" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="G36" s="16" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
+      <c r="E36" s="16" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="16" t="n">
+        <v>2</v>
       </c>
       <c r="H36" s="16" t="inlineStr">
         <is>
@@ -6701,7 +6689,7 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>Maximum extrapolation duration beyond pose_max_age</t>
+          <t>CORNER_ALIGN dwell: heading+yaw-rate must both be stable this long before exit→TRACK (BUG-T1 036f116)</t>
         </is>
       </c>
     </row>
@@ -6713,12 +6701,12 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Feedforward YR (P3.1)</t>
+          <t>Latency (P2.4)</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>use_feedforward_yaw_rate</t>
+          <t>use_imu_extrapolation</t>
         </is>
       </c>
       <c r="D37" s="15" t="inlineStr">
@@ -6728,7 +6716,7 @@
       </c>
       <c r="E37" s="15" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="F37" s="15" t="inlineStr">
@@ -6748,7 +6736,7 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>Enable ω = κ·v + k_ψ·θ_e yaw rate output</t>
+          <t>Enable velocity-based pose extrapolation</t>
         </is>
       </c>
     </row>
@@ -6760,12 +6748,12 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Feedforward YR (P3.1)</t>
+          <t>Latency (P2.4)</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>yaw_rate_feedback_gain</t>
+          <t>imu_max_extrap_age_s</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
@@ -6775,27 +6763,27 @@
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
+        <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="F38" s="16" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
       <c r="G38" s="16" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="H38" s="16" t="inlineStr">
         <is>
-          <t>rad/s/rad</t>
+          <t>s</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Heading error feedback term k_ψ</t>
+          <t>Maximum extrapolation duration beyond pose_max_age</t>
         </is>
       </c>
     </row>
@@ -6812,131 +6800,131 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
+          <t>use_feedforward_yaw_rate</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Enable ω = κ·v + k_ψ·θ_e yaw rate output</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="50" customHeight="1">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>RPP Controller</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Feedforward YR (P3.1)</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>yaw_rate_feedback_gain</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>rad/s/rad</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Heading error feedback term k_ψ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="23" t="inlineStr">
+        <is>
+          <t>RPP Controller</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Feedforward YR (P3.1)</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
           <t>max_yaw_rate_body</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E39" s="15" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
         <is>
           <t>0.45</t>
         </is>
       </c>
-      <c r="F39" s="15" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="G39" s="15" t="inlineStr">
+      <c r="G41" s="15" t="inlineStr">
         <is>
           <t>5.0</t>
         </is>
       </c>
-      <c r="H39" s="15" t="inlineStr">
+      <c r="H41" s="15" t="inlineStr">
         <is>
           <t>rad/s</t>
         </is>
       </c>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>Body yaw rate clamp (≈57°/s at 1.0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="50" customHeight="1">
-      <c r="A40" s="26" t="inlineStr">
-        <is>
-          <t>Spray Controller</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Actuator</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>actuator_set_index</t>
-        </is>
-      </c>
-      <c r="D40" s="16" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="E40" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F40" s="16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G40" s="16" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H40" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Which Actuator Set param carries ON/OFF signal</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="50" customHeight="1">
-      <c r="A41" s="26" t="inlineStr">
-        <is>
-          <t>Spray Controller</t>
-        </is>
-      </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>Actuator</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
-        <is>
-          <t>on_value</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="F41" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G41" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="inlineStr">
-        <is>
-          <t>+1.0 → MAX PWM → solenoid ON</t>
         </is>
       </c>
     </row>
@@ -6953,37 +6941,37 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>off_value</t>
+          <t>actuator_set_index</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>-1.0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G42" s="16" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H42" s="16" t="inlineStr">
+        <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G42" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>-1.0 → MIN PWM → solenoid OFF</t>
+          <t>Which Actuator Set param carries ON/OFF signal</t>
         </is>
       </c>
     </row>
@@ -6995,22 +6983,22 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Actuator</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>debounce_samples</t>
+          <t>on_value</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F43" s="15" t="inlineStr">
@@ -7025,12 +7013,12 @@
       </c>
       <c r="H43" s="15" t="inlineStr">
         <is>
-          <t>samples</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>≈60ms at 50Hz — prevent chatter on rapid transitions</t>
+          <t>+1.0 → MAX PWM → solenoid ON</t>
         </is>
       </c>
     </row>
@@ -7042,12 +7030,12 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Actuator</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>reassert_hz</t>
+          <t>off_value</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
@@ -7057,7 +7045,7 @@
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>-1.0</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
@@ -7072,12 +7060,12 @@
       </c>
       <c r="H44" s="16" t="inlineStr">
         <is>
-          <t>Hz</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>Re-send desired spray state to compensate dropped commands</t>
+          <t>-1.0 → MIN PWM → solenoid OFF</t>
         </is>
       </c>
     </row>
@@ -7094,17 +7082,17 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>require_offboard</t>
+          <t>debounce_samples</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F45" s="15" t="inlineStr">
@@ -7119,12 +7107,12 @@
       </c>
       <c r="H45" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>samples</t>
         </is>
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>Only spray when FCU mode = OFFBOARD</t>
+          <t>≈60ms at 50Hz — prevent chatter on rapid transitions</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7129,7 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>active_timeout_s</t>
+          <t>reassert_hz</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
@@ -7151,7 +7139,7 @@
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
@@ -7166,12 +7154,12 @@
       </c>
       <c r="H46" s="16" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Hz</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>Force OFF if /spray/active goes stale beyond this</t>
+          <t>Re-send desired spray state to compensate dropped commands</t>
         </is>
       </c>
     </row>
@@ -7188,131 +7176,131 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
+          <t>require_offboard</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F47" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>Only spray when FCU mode = OFFBOARD</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="50" customHeight="1">
+      <c r="A48" s="26" t="inlineStr">
+        <is>
+          <t>Spray Controller</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>active_timeout_s</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Force OFF if /spray/active goes stale beyond this</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="A49" s="26" t="inlineStr">
+        <is>
+          <t>Spray Controller</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
           <t>manual_override_timeout_s</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E47" s="15" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>10.0</t>
         </is>
       </c>
-      <c r="F47" s="15" t="inlineStr">
+      <c r="F49" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G47" s="15" t="inlineStr">
+      <c r="G49" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H47" s="15" t="inlineStr">
+      <c r="H49" s="15" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="I47" s="7" t="inlineStr">
+      <c r="I49" s="7" t="inlineStr">
         <is>
           <t>Hard expiry on manual bench-test ON command</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="50" customHeight="1">
-      <c r="A48" s="24" t="inlineStr">
-        <is>
-          <t>Server Config</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>Telemetry</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>TELEMETRY_HZ</t>
-        </is>
-      </c>
-      <c r="D48" s="16" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="E48" s="16" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="F48" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G48" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="16" t="inlineStr">
-        <is>
-          <t>Hz</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
-        <is>
-          <t>WebSocket telemetry push rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="50" customHeight="1">
-      <c r="A49" s="24" t="inlineStr">
-        <is>
-          <t>Server Config</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>POSE_STALE_MS</t>
-        </is>
-      </c>
-      <c r="D49" s="15" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="E49" s="15" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="F49" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="15" t="inlineStr">
-        <is>
-          <t>ms</t>
-        </is>
-      </c>
-      <c r="I49" s="7" t="inlineStr">
-        <is>
-          <t>Pose staleness threshold for server-side watchdog</t>
         </is>
       </c>
     </row>
@@ -7324,22 +7312,22 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Telemetry</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>SAFETY_STALE_GRACE_S</t>
+          <t>TELEMETRY_HZ</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
@@ -7354,12 +7342,12 @@
       </c>
       <c r="H50" s="16" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Hz</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
         <is>
-          <t>Abort after sustained stale beyond this grace period</t>
+          <t>WebSocket telemetry push rate</t>
         </is>
       </c>
     </row>
@@ -7371,22 +7359,22 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Mission</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>DONE_SETTLE_S</t>
+          <t>POSE_STALE_MS</t>
         </is>
       </c>
       <c r="D51" s="15" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="E51" s="15" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>500</t>
         </is>
       </c>
       <c r="F51" s="15" t="inlineStr">
@@ -7401,12 +7389,12 @@
       </c>
       <c r="H51" s="15" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>ms</t>
         </is>
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>Require 1s in DONE state before declaring mission complete</t>
+          <t>Pose staleness threshold for server-side watchdog</t>
         </is>
       </c>
     </row>
@@ -7418,12 +7406,12 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Spray</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>SPRAY_LITERS_PER_METER</t>
+          <t>SAFETY_STALE_GRACE_S</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
@@ -7433,7 +7421,7 @@
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>0.012</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
@@ -7448,12 +7436,12 @@
       </c>
       <c r="H52" s="16" t="inlineStr">
         <is>
-          <t>L/m</t>
+          <t>s</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
         <is>
-          <t>Marking fluid consumption rate (env-tunable)</t>
+          <t>Abort after sustained stale beyond this grace period</t>
         </is>
       </c>
     </row>
@@ -7465,22 +7453,22 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Spray</t>
+          <t>Mission</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>MAX_SPRAY_TEST_DURATION_S</t>
+          <t>DONE_SETTLE_S</t>
         </is>
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E53" s="15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F53" s="15" t="inlineStr">
@@ -7500,7 +7488,7 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>Max duration for manual spray bench test</t>
+          <t>Require 1s in DONE state before declaring mission complete</t>
         </is>
       </c>
     </row>
@@ -7512,12 +7500,12 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>Spray</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>RMSE_MAX</t>
+          <t>SPRAY_LITERS_PER_METER</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
@@ -7527,7 +7515,7 @@
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
-          <t>0.05</t>
+          <t>0.012</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
@@ -7542,12 +7530,12 @@
       </c>
       <c r="H54" s="16" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>L/m</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
         <is>
-          <t>DXF→NED alignment RMSE quality gate</t>
+          <t>Marking fluid consumption rate (env-tunable)</t>
         </is>
       </c>
     </row>
@@ -7559,136 +7547,136 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
+          <t>Spray</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>MAX_SPRAY_TEST_DURATION_S</t>
+        </is>
+      </c>
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F55" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>Max duration for manual spray bench test</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="50" customHeight="1">
+      <c r="A56" s="24" t="inlineStr">
+        <is>
+          <t>Server Config</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
           <t>Planning</t>
         </is>
       </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>RMSE_MAX</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="16" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>DXF→NED alignment RMSE quality gate</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="50" customHeight="1">
+      <c r="A57" s="24" t="inlineStr">
+        <is>
+          <t>Server Config</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Planning</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
         <is>
           <t>STAGING_TTL_S</t>
         </is>
       </c>
-      <c r="D55" s="15" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="E55" s="15" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>3600</t>
         </is>
       </c>
-      <c r="F55" s="15" t="inlineStr">
+      <c r="F57" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G55" s="15" t="inlineStr">
+      <c r="G57" s="15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H55" s="15" t="inlineStr">
+      <c r="H57" s="15" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="I55" s="7" t="inlineStr">
+      <c r="I57" s="7" t="inlineStr">
         <is>
           <t>Staged mission lifetime before expiry</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="50" customHeight="1">
-      <c r="A56" s="27" t="inlineStr">
-        <is>
-          <t>Path Engine</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>Discretization</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>line_spacing</t>
-        </is>
-      </c>
-      <c r="D56" s="16" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E56" s="16" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="F56" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G56" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H56" s="16" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
-        <is>
-          <t>MARK segment waypoint spacing</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="50" customHeight="1">
-      <c r="A57" s="27" t="inlineStr">
-        <is>
-          <t>Path Engine</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>Discretization</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>transit_spacing</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="E57" s="15" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="F57" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G57" s="15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H57" s="15" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="I57" s="7" t="inlineStr">
-        <is>
-          <t>TRANSIT segment waypoint spacing</t>
         </is>
       </c>
     </row>
@@ -7700,12 +7688,12 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>Velocity</t>
+          <t>Discretization</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>marking_speed</t>
+          <t>line_spacing</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
@@ -7715,7 +7703,7 @@
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
@@ -7730,12 +7718,12 @@
       </c>
       <c r="H58" s="16" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>m</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
         <is>
-          <t>Speed during MARK segments</t>
+          <t>MARK segment waypoint spacing</t>
         </is>
       </c>
     </row>
@@ -7747,12 +7735,12 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Velocity</t>
+          <t>Discretization</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>transit_speed</t>
+          <t>transit_spacing</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">
@@ -7762,7 +7750,7 @@
       </c>
       <c r="E59" s="15" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="F59" s="15" t="inlineStr">
@@ -7777,12 +7765,12 @@
       </c>
       <c r="H59" s="15" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>m</t>
         </is>
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>Speed during TRANSIT repositioning segments</t>
+          <t>TRANSIT segment waypoint spacing</t>
         </is>
       </c>
     </row>
@@ -7794,22 +7782,22 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Extensions</t>
+          <t>Velocity</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>enable_path_extensions</t>
+          <t>marking_speed</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>0.35</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
@@ -7824,12 +7812,12 @@
       </c>
       <c r="H60" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>m/s</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
         <is>
-          <t>Enable pre/aft spray lead-in/out extension</t>
+          <t>Speed during MARK segments</t>
         </is>
       </c>
     </row>
@@ -7841,12 +7829,12 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Extensions</t>
+          <t>Velocity</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>pre_extension_m</t>
+          <t>transit_speed</t>
         </is>
       </c>
       <c r="D61" s="15" t="inlineStr">
@@ -7856,7 +7844,7 @@
       </c>
       <c r="E61" s="15" t="inlineStr">
         <is>
-          <t>0.035</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="F61" s="15" t="inlineStr">
@@ -7871,12 +7859,12 @@
       </c>
       <c r="H61" s="15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m/s</t>
         </is>
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>Lead-in distance before MARK segment starts</t>
+          <t>Speed during TRANSIT repositioning segments</t>
         </is>
       </c>
     </row>
@@ -7893,35 +7881,129 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
+          <t>enable_path_extensions</t>
+        </is>
+      </c>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G62" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>Enable pre/aft spray lead-in/out extension</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="27" t="inlineStr">
+        <is>
+          <t>Path Engine</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Extensions</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>pre_extension_m</t>
+        </is>
+      </c>
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="E63" s="15" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H63" s="15" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>Lead-in distance before MARK segment starts</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="27" t="inlineStr">
+        <is>
+          <t>Path Engine</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Extensions</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
           <t>aft_extension_m</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr">
+      <c r="D64" s="16" t="inlineStr">
         <is>
           <t>float</t>
         </is>
       </c>
-      <c r="E62" s="16" t="inlineStr">
+      <c r="E64" s="16" t="inlineStr">
         <is>
           <t>0.0035</t>
         </is>
       </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="F64" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G62" s="16" t="inlineStr">
+      <c r="G64" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H62" s="16" t="inlineStr">
+      <c r="H64" s="16" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="I62" s="4" t="inlineStr">
+      <c r="I64" s="4" t="inlineStr">
         <is>
           <t>Lead-out distance after MARK segment ends</t>
         </is>
@@ -7965,7 +8047,7 @@
       </c>
       <c r="C1" s="39" t="inlineStr">
         <is>
-          <t>Total: 34 | open ~18 | 3 bug-fix + PE-T4/T5 validation</t>
+          <t>Total:34 | BUG-T3 done; BUG-T1/T2 committed→validating</t>
         </is>
       </c>
     </row>
@@ -9097,7 +9179,7 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Validating</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -9112,7 +9194,7 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>Hypothesis: align-phase yaw-rate limit-cycle near v≈0 (rate-loop P/I with no deadband) and/or RO_YAW_RATE_I windup. Check pivot entry/exit gating + segment_heading_tolerance_deg.</t>
+          <t>FIX COMMITTED 036f116 (yaw-rate settle gates: CORNER_STOP joint speed+yaw-rate AND-gate; CORNER_ALIGN exit needs heading+yaw-rate stable for segment_align_settle_s=0.10s; new params segment_stop_yaw_rate_threshold=0.05). NOTE: Opus's 'RO_YAW_RATE_LIM 90→35' action is MOOT — already 30 (validated log_183). Pending bag validation.</t>
         </is>
       </c>
     </row>
@@ -9134,7 +9216,7 @@
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Validating</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -9149,7 +9231,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Hypothesis: per-entity run splitter inserts a stop/align transition even when junction angle≈0. Check segment_corner_threshold_deg gating + run-transition logic + tracking_profile=auto entity boundaries.</t>
+          <t>FIX COMMITTED 1af51ac — hard stops at smooth run/segment boundaries. Pending bag validation (confirm continuous flow across tangent junctions).</t>
         </is>
       </c>
     </row>
@@ -9171,7 +9253,7 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -9186,7 +9268,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Hypothesis: angle-wrap/sign bug on the large initial heading error OR negative-speed projection making PX4 pick the 180° solution (OFFBOARD bug #2/#3 lineage). HIGH SAFETY relevance.</t>
+          <t>DONE 2026-06-13 (opus) commit 510be9b — forward-cone clamp on first-segment velocity. Deployed: FF pull, rpp-pipeline restart (2s, MAVROS intact), 3/3 services active, API ping OK. Mac==origin==Jetson.</t>
         </is>
       </c>
     </row>

</xml_diff>